<commit_message>
Force update of YAML
</commit_message>
<xml_diff>
--- a/battery_report_2025-12-12.xlsx
+++ b/battery_report_2025-12-12.xlsx
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025-12-12T01:58:28.471358</t>
+          <t>2025-12-12T03:31:10.663532</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -499,7 +499,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T01:58:28.471604</t>
+          <t>2025-12-12T03:31:10.663820</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -526,7 +526,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T01:58:28.471639</t>
+          <t>2025-12-12T03:31:10.663903</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T01:58:28.471702</t>
+          <t>2025-12-12T03:31:10.663981</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -580,7 +580,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T01:58:28.471791</t>
+          <t>2025-12-12T03:31:10.664068</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
update on checking clicks on notification
</commit_message>
<xml_diff>
--- a/battery_report_2025-12-12.xlsx
+++ b/battery_report_2025-12-12.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detailed Logs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+        <bgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,13 +74,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,6 +473,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>User_Action</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
@@ -472,7 +485,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025-12-12T03:31:10.663532</t>
+          <t>2025-12-12T03:59:39.122290</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -491,6 +504,11 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Orphan Lock - No User Mapping Found</t>
         </is>
@@ -499,7 +517,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T03:31:10.663820</t>
+          <t>2025-12-12T03:59:39.122697</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -519,88 +537,190 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>OPENED</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12T03:31:10.663903</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-12T03:59:39.122849</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>L102</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>U_C</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>NO_RESPONSE</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12T03:31:10.663981</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-12T03:59:39.122989</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>L104</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>U_E</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>NO_RESPONSE</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12T03:31:10.664068</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-12T03:59:39.123202</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>L105</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>U_A</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>NO_RESPONSE</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Campaign Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Campaign ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>battery_check_2025_W49</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Notifications Sent</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Total User Clicks</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Click Through Rate (CTR)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>25.00%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated effectiveness and readme
</commit_message>
<xml_diff>
--- a/battery_report_2025-12-12.xlsx
+++ b/battery_report_2025-12-12.xlsx
@@ -45,14 +45,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFFCC"/>
+        <bgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor rgb="00FFFFCC"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +478,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
@@ -485,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025-12-12T03:59:39.122290</t>
+          <t>2025-12-12T04:09:40.431042</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -509,6 +514,11 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Orphan Lock - No User Mapping Found</t>
         </is>
@@ -517,7 +527,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2025-12-12T03:59:39.122697</t>
+          <t>2025-12-12T04:09:40.431301</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -537,10 +547,15 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>OPENED</t>
+          <t>NO_RESPONSE</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>EFFECTIVE</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
@@ -549,7 +564,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2025-12-12T03:59:39.122849</t>
+          <t>2025-12-12T04:09:40.431397</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -569,42 +584,52 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>OPENED</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-12T04:09:40.431492</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>L104</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>U_E</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>NO_RESPONSE</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2025-12-12T03:59:39.122989</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>L104</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>U_E</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>NO_RESPONSE</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
@@ -613,7 +638,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2025-12-12T03:59:39.123202</t>
+          <t>2025-12-12T04:09:40.431587</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -633,10 +658,15 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>NO_RESPONSE</t>
+          <t>OPENED</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Notification Sent (Campgn: battery_check_2025_W49)</t>
         </is>
@@ -653,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,22 +735,36 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total User Clicks</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
+          <t>User Clicks (CTR)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2 (50.0%)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Click Through Rate (CTR)</t>
+          <t>Effective Conversions</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>1 (25.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Effectiveness = Users who updated lock timestamp</t>
         </is>
       </c>
     </row>

</xml_diff>